<commit_message>
feat: add client-side Excel-based portfolio user and password services and seed data
</commit_message>
<xml_diff>
--- a/client/public/portfolio_data.xlsx
+++ b/client/public/portfolio_data.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Skills" sheetId="4" r:id="rId4"/>
     <sheet name="Education" sheetId="5" r:id="rId5"/>
     <sheet name="Achievements" sheetId="6" r:id="rId6"/>
+    <sheet name="Admin" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -1395,4 +1396,37 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Username</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Password</v>
+      </c>
+      <c r="C1" t="str">
+        <v>UpdatedAt</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>admin</v>
+      </c>
+      <c r="B2" t="str">
+        <v>admin@portfolio2026</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-09-18T09:11:38.894Z</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>